<commit_message>
ops(comp): base is a retainer against 15-20 hr/wk engagement, not a 10-hr wage
Expected engagement 15-20 hrs/week (internship-level); base-only reads
$10/hr with fairness judged at target total comp (~$13/hr target,
$15+/hr stretch). Scenario hours updated to 15/18/20.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QGYDg6ZViFFeNuPbg8Zoy8
</commit_message>
<xml_diff>
--- a/10-ops/gtm-role-comp-program-v4.xlsx
+++ b/10-ops/gtm-role-comp-program-v4.xlsx
@@ -561,7 +561,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>3. Fairness floor: base + realistic variable should clear ~$15/hr for committed hours (see Scenarios hourly check).</t>
+          <t>3. Fairness check: base alone is a retainer, deliberately below market; TOTAL comp at target productivity should clear ~$13–15/hr (see Scenarios hourly check).</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Committed floor: 10 hrs/week (base covers this). Typical: 15–20.</t>
+          <t>Expected engagement: 15–20 hrs/week (internship-level commitment;</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -757,7 +757,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Owns:</t>
+          <t xml:space="preserve">  the base is a retainer — variable comp is what pays the hours).</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • List building in approved lanes only</t>
+          <t>Owns:</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Personalized outreach — every send individually researched;</t>
+          <t xml:space="preserve">  • List building in approved lanes only</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -793,7 +793,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    first 2 weeks of sends reviewed before sending</t>
+          <t xml:space="preserve">  • Personalized outreach — every send individually researched;</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -805,7 +805,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Follow-up sequences (touches 2–4) — most replies live here</t>
+          <t xml:space="preserve">    first 2 weeks of sends reviewed before sending</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -817,7 +817,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Booking + meeting prep; same-day notes to founder</t>
+          <t xml:space="preserve">  • Follow-up sequences (touches 2–4) — most replies live here</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -829,7 +829,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Daily end-of-day tracker (see Daily_Tracker)</t>
+          <t xml:space="preserve">  • Booking + meeting prep; same-day notes to founder</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -841,7 +841,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Does NOT own:</t>
+          <t xml:space="preserve">  • Daily end-of-day tracker (see Daily_Tracker)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -853,7 +853,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Closing (founder closes), pricing, discounts</t>
+          <t>Does NOT own:</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -865,7 +865,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Choosing new ICPs / verticals — written approval first</t>
+          <t xml:space="preserve">  • Closing (founder closes), pricing, discounts</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -877,7 +877,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Content production</t>
+          <t xml:space="preserve">  • Choosing new ICPs / verticals — written approval first</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -889,12 +889,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Content production</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Compensation: Content_Comp tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Compensation: SDR_Comp tab.</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Compensation: Content_Comp tab.</t>
         </is>
       </c>
     </row>
@@ -956,38 +963,38 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Guaranteed. Covers the 10 hr/week committed floor.</t>
+          <t>A guaranteed retainer — NOT an hourly wage. Variable comp is where the hours pay off.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Committed hours/week (floor)</t>
+          <t>Expected engagement (hrs/week)</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Below this two weeks running → base pro-rates.</t>
+          <t>Internship-level commitment: 15–20 typical. Visibly below this two weeks running → base pro-rates.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Implied floor rate ($/hr)</t>
+          <t>Base-only equivalent ($/hr)</t>
         </is>
       </c>
       <c r="B7" s="11">
         <f>B5/(B6*52/12)</f>
         <v/>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Fairness check: keep ≥ ~$15/hr.</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Deliberately below market on its own. Fairness is judged at TARGET total comp (Scenarios): ~$13/hr target, $15+/hr stretch.</t>
         </is>
       </c>
     </row>
@@ -1774,10 +1781,10 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>20</v>
@@ -1879,7 +1886,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Fairness check: hourly equivalent should stay ≥ ~$15/hr at every level.</t>
+          <t>Fairness check: total comp ≈ $13/hr at TARGET and $15+/hr at STRETCH. Base alone is a retainer, not the wage — output closes the gap.</t>
         </is>
       </c>
     </row>

</xml_diff>